<commit_message>
bản cập nhật an toàn, chạy ổn với testcase cơ bản login, register
</commit_message>
<xml_diff>
--- a/product Tester/templates/test-cases-test.xlsx
+++ b/product Tester/templates/test-cases-test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="18251" windowHeight="8255"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -1046,7 +1046,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3192780" y="3773805"/>
+          <a:off x="3192780" y="3764280"/>
           <a:ext cx="243840" cy="243840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1396,7 +1396,7 @@
     <col min="6" max="6" width="27.3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.35" spans="1:5">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1603,7 +1603,7 @@
       <c r="C25" s="10"/>
       <c r="D25" s="8"/>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" ht="16.35" spans="1:4">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="C26" s="11"/>
@@ -1623,7 +1623,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" ht="16.35" spans="1:4">
       <c r="A28" s="12"/>
       <c r="B28" s="13"/>
       <c r="C28" s="10"/>

</xml_diff>